<commit_message>
PDF y Excel: tabla blanca en hoja 1, tabla verde CPA en hoja 2
El resumen queda con fondo blanco en la primera hoja. Los 15 puntos
CPA control van en una tabla verde propia, en la segunda hoja.

Co-authored-by: anibaloperacionesWes <anibaloperacionesWes@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/Usuarios/acceso_por_empresa/accesos_por_empresa.xlsx
+++ b/reports/Usuarios/acceso_por_empresa/accesos_por_empresa.xlsx
@@ -8,45 +8,47 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Puntos" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="000020 AGUNSA" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="000021 CDUC" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="000031 Club Providencia" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="000009 COPEC" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="000008 CORMUP" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="000010 Corporación Puente Alto" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="000012 DERCO" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="000027 Fundo Zapallar" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="000028 La Florida" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="000024 La Reina" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="000022 Las Condes" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="000002 Lo valledor" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="000007 Nido de Aguilas" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="000025 Parque Arauco" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="000006 Providencia" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="000017 Renca" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="000026 UDD" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CPA control" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Puntos" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="000020 AGUNSA" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="000021 CDUC" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="000031 Club Providencia" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="000009 COPEC" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="000008 CORMUP" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="000010 Corporación Puente Alto" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="000012 DERCO" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="000027 Fundo Zapallar" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="000028 La Florida" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="000024 La Reina" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="000022 Las Condes" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="000002 Lo valledor" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="000007 Nido de Aguilas" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="000025 Parque Arauco" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="000006 Providencia" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="000017 Renca" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="000026 UDD" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$4:$I$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Puntos'!$A$4:$F$115</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'000020 AGUNSA'!$A$4:$H$19</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'000021 CDUC'!$A$4:$H$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'000031 Club Providencia'!$A$4:$H$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'000009 COPEC'!$A$4:$H$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'000008 CORMUP'!$A$4:$H$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'000010 Corporación Puente Alto'!$A$4:$H$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'000012 DERCO'!$A$4:$H$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'000027 Fundo Zapallar'!$A$4:$H$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'000028 La Florida'!$A$4:$H$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'000024 La Reina'!$A$4:$H$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'000022 Las Condes'!$A$4:$H$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'000002 Lo valledor'!$A$4:$H$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'000007 Nido de Aguilas'!$A$4:$H$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'000025 Parque Arauco'!$A$4:$H$29</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'000006 Providencia'!$A$4:$H$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'000017 Renca'!$A$4:$H$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'000026 UDD'!$A$4:$H$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CPA control'!$A$4:$F$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Puntos'!$A$4:$F$115</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'000020 AGUNSA'!$A$4:$H$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'000021 CDUC'!$A$4:$H$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'000031 Club Providencia'!$A$4:$H$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'000009 COPEC'!$A$4:$H$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'000008 CORMUP'!$A$4:$H$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'000010 Corporación Puente Alto'!$A$4:$H$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'000012 DERCO'!$A$4:$H$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'000027 Fundo Zapallar'!$A$4:$H$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'000028 La Florida'!$A$4:$H$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'000024 La Reina'!$A$4:$H$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'000022 Las Condes'!$A$4:$H$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'000002 Lo valledor'!$A$4:$H$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'000007 Nido de Aguilas'!$A$4:$H$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'000025 Parque Arauco'!$A$4:$H$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'000006 Providencia'!$A$4:$H$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'000017 Renca'!$A$4:$H$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'000026 UDD'!$A$4:$H$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -55,7 +57,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -72,8 +74,13 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00375623"/>
+      <sz val="14"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -95,6 +102,11 @@
         <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00375623"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -108,7 +120,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -117,6 +129,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -571,10 +585,10 @@
       <c r="C5" t="n">
         <v>5</v>
       </c>
-      <c r="D5" s="3" t="n">
+      <c r="D5" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="E5" t="n">
         <v>4</v>
       </c>
       <c r="F5" t="n">
@@ -610,10 +624,10 @@
       <c r="C6" t="n">
         <v>5</v>
       </c>
-      <c r="D6" s="3" t="n">
+      <c r="D6" t="n">
         <v>2</v>
       </c>
-      <c r="E6" s="4" t="n">
+      <c r="E6" t="n">
         <v>3</v>
       </c>
       <c r="F6" t="n">
@@ -652,7 +666,7 @@
       <c r="D7" t="n">
         <v>0</v>
       </c>
-      <c r="E7" s="4" t="n">
+      <c r="E7" t="n">
         <v>2</v>
       </c>
       <c r="F7" t="n">
@@ -687,7 +701,7 @@
       <c r="D8" t="n">
         <v>0</v>
       </c>
-      <c r="E8" s="4" t="n">
+      <c r="E8" t="n">
         <v>11</v>
       </c>
       <c r="F8" t="n">
@@ -719,10 +733,10 @@
       <c r="C9" t="n">
         <v>14</v>
       </c>
-      <c r="D9" s="3" t="n">
+      <c r="D9" t="n">
         <v>4</v>
       </c>
-      <c r="E9" s="4" t="n">
+      <c r="E9" t="n">
         <v>10</v>
       </c>
       <c r="F9" t="n">
@@ -761,7 +775,7 @@
       <c r="D10" t="n">
         <v>0</v>
       </c>
-      <c r="E10" s="4" t="n">
+      <c r="E10" t="n">
         <v>11</v>
       </c>
       <c r="F10" t="n">
@@ -796,7 +810,7 @@
       <c r="D11" t="n">
         <v>0</v>
       </c>
-      <c r="E11" s="4" t="n">
+      <c r="E11" t="n">
         <v>7</v>
       </c>
       <c r="F11" t="n">
@@ -831,7 +845,7 @@
       <c r="D12" t="n">
         <v>0</v>
       </c>
-      <c r="E12" s="4" t="n">
+      <c r="E12" t="n">
         <v>8</v>
       </c>
       <c r="F12" t="n">
@@ -863,7 +877,7 @@
       <c r="C13" t="n">
         <v>1</v>
       </c>
-      <c r="D13" s="3" t="n">
+      <c r="D13" t="n">
         <v>1</v>
       </c>
       <c r="E13" t="n">
@@ -898,7 +912,7 @@
       <c r="C14" t="n">
         <v>1</v>
       </c>
-      <c r="D14" s="3" t="n">
+      <c r="D14" t="n">
         <v>1</v>
       </c>
       <c r="E14" t="n">
@@ -936,7 +950,7 @@
       <c r="D15" t="n">
         <v>0</v>
       </c>
-      <c r="E15" s="4" t="n">
+      <c r="E15" t="n">
         <v>1</v>
       </c>
       <c r="F15" t="n">
@@ -968,10 +982,10 @@
       <c r="C16" t="n">
         <v>2</v>
       </c>
-      <c r="D16" s="3" t="n">
+      <c r="D16" t="n">
         <v>1</v>
       </c>
-      <c r="E16" s="4" t="n">
+      <c r="E16" t="n">
         <v>1</v>
       </c>
       <c r="F16" t="n">
@@ -1010,7 +1024,7 @@
       <c r="D17" t="n">
         <v>0</v>
       </c>
-      <c r="E17" s="4" t="n">
+      <c r="E17" t="n">
         <v>7</v>
       </c>
       <c r="F17" t="n">
@@ -1042,10 +1056,10 @@
       <c r="C18" t="n">
         <v>25</v>
       </c>
-      <c r="D18" s="3" t="n">
+      <c r="D18" t="n">
         <v>3</v>
       </c>
-      <c r="E18" s="4" t="n">
+      <c r="E18" t="n">
         <v>22</v>
       </c>
       <c r="F18" t="n">
@@ -1084,7 +1098,7 @@
       <c r="D19" t="n">
         <v>0</v>
       </c>
-      <c r="E19" s="4" t="n">
+      <c r="E19" t="n">
         <v>4</v>
       </c>
       <c r="F19" t="n">
@@ -1116,10 +1130,10 @@
       <c r="C20" t="n">
         <v>5</v>
       </c>
-      <c r="D20" s="3" t="n">
+      <c r="D20" t="n">
         <v>2</v>
       </c>
-      <c r="E20" s="4" t="n">
+      <c r="E20" t="n">
         <v>3</v>
       </c>
       <c r="F20" t="n">
@@ -1158,7 +1172,7 @@
       <c r="D21" t="n">
         <v>0</v>
       </c>
-      <c r="E21" s="4" t="n">
+      <c r="E21" t="n">
         <v>2</v>
       </c>
       <c r="F21" t="n">
@@ -1187,6 +1201,139 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="70" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>DERCO (000012)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1 usuario(s) · 7 punto(s) activo(s) · 0 CPA · 7 solo monitoreo</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>CPA: —  |  Solo monitoreo: 000012-06, 000012-07, 000012-08, 000012-09, 000012-10, 000012-11, 000012-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Nombre</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Cuenta de esta empresa</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Empresa de la cuenta</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Switch on/off</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Puntos con acceso</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Node IDs</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Puntos (nombre)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>go.salass@gmail.com</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Gonzalo Salas</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Wes Spa</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>000012-06, 000012-07, 000012-08, 000012-09, 000012-10, 000012-11, 000012-12</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>000012-06 (Quilicura Matriz Principal); 000012-07 (Quilicura Dercomaq); 000012-08 (Quilicura Lav. de Maquinas); 000012-09 (Quilicura Casino); 000012-10 (Quilicura Proderco); 000012-11 (Quilicura Camarines); 000012-12 (Quilicura Edificio JCB)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:H5"/>
+  <mergeCells count="3">
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1559,7 +1706,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1692,7 +1839,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1865,7 +2012,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1998,7 +2145,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2331,7 +2478,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2584,7 +2731,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3677,7 +3824,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4250,7 +4397,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4383,7 +4530,560 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Puntos CPA control (monitoreo con control)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Hoja 2 · sitios con horario programado en «Horarios de contron hidrico clientes wes» (Drive).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>node_id</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>nombre</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>company_id</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>empresa</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>tipo</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>nombre_en_excel_horarios</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>000020-02</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Modulo D</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>000020</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>AGUNSA</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>CPA (monitoreo con control)</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>agunsa modulo d</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>000021-01</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Club House CDUC</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>000021</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>CDUC</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>CPA (monitoreo con control)</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>club hause UC</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>000021-03</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Raimundo Tupper</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>000021</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>CDUC</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>CPA (monitoreo con control)</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>raymundo tupper</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>000008-01</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Lic. Antonio Hermida F</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>000008</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>CORMUP</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>CPA (monitoreo con control)</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>171 antonio hermidas fabres</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>000008-03</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Carlos Fernandez P.</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>000008</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>CORMUP</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>CPA (monitoreo con control)</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>carlos fernandes peña</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>000008-04</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Tobalaba</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>000008</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>CORMUP</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>CPA (monitoreo con control)</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>colegio tobalaba</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>000008-05</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Santa Maria</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>000008</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>CORMUP</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>CPA (monitoreo con control)</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>colegio santa maria</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>000028-01</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Liceo Alto Cordillera</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>000028</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>La Florida</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>CPA (monitoreo con control)</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>liceo alto cordillera la florida</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>000024-01</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Eugenio María De Hostos</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>000024</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>La Reina</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>CPA (monitoreo con control)</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>eugenio maria de hostos</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>000002-01</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Lo Valledor - P1</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>000002</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Lo valledor</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>CPA (monitoreo con control)</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>lo valledor p1</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>000025-01</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Estanque Norte Locales Mall</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>000025</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Parque Arauco</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>CPA (monitoreo con control)</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>PAE estanquer norte locales</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>000025-07</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>PIZZA HUT</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>000025</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Parque Arauco</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>CPA (monitoreo con control)</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>pizza hut</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>000025-19</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Sala de Bomba Estanque Sur</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>000025</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Parque Arauco</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>CPA (monitoreo con control)</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>mae  sala de bomba estanque sur</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>000017-07</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Cumbre de cóndores pte.</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>000017</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Renca</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>CPA (monitoreo con control)</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>ICCP</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>000017-08</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Cumbre de cóndores Ote.</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>000017</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Renca</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>CPA (monitoreo con control)</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>ICCO</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:F19"/>
+  <mergeCells count="2">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4556,7 +5256,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4645,7 +5345,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -4705,7 +5404,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4733,7 +5431,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -4761,7 +5458,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4853,7 +5549,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -4881,7 +5576,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4909,7 +5603,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -4937,7 +5630,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -4965,7 +5657,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -4993,7 +5684,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -5021,7 +5711,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -5049,7 +5738,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -5077,7 +5765,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -5105,7 +5792,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -5133,7 +5819,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -5161,7 +5846,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -5189,7 +5873,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -5217,7 +5900,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -5245,7 +5927,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -5273,7 +5954,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -5333,7 +6013,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -5457,7 +6136,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -5485,7 +6163,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -5513,7 +6190,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -5541,7 +6217,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -5569,7 +6244,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -5597,7 +6271,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -5625,7 +6298,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -5653,7 +6325,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -5681,7 +6352,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -5709,7 +6379,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -5737,7 +6406,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -5765,7 +6433,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -5793,7 +6460,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -5821,7 +6487,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -5849,7 +6514,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -5877,7 +6541,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -5905,7 +6568,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -5933,7 +6595,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -5961,7 +6622,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -5989,7 +6649,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -6017,7 +6676,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -6045,7 +6703,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -6073,7 +6730,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -6101,7 +6757,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -6129,7 +6784,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -6157,7 +6811,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -6185,7 +6838,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -6213,7 +6865,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -6241,7 +6892,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -6269,7 +6919,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -6297,7 +6946,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -6325,7 +6973,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -6353,7 +7000,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -6381,7 +7027,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -6409,7 +7054,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -6501,7 +7145,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -6561,7 +7204,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -6589,7 +7231,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -6617,7 +7258,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -6645,7 +7285,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -6673,7 +7312,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -6701,7 +7339,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -6729,7 +7366,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -6757,7 +7393,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -6817,7 +7452,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -6877,7 +7511,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -6905,7 +7538,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -6933,7 +7565,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -6961,7 +7592,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -6989,7 +7619,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -7017,7 +7646,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -7077,7 +7705,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -7105,7 +7732,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -7133,7 +7759,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -7161,7 +7786,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -7189,7 +7813,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -7217,7 +7840,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -7245,7 +7867,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -7273,7 +7894,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -7301,7 +7921,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -7329,7 +7948,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -7357,7 +7975,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -7385,7 +8002,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -7413,7 +8029,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -7441,7 +8056,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -7469,7 +8083,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -7497,7 +8110,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -7525,7 +8137,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -7553,7 +8164,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -7581,7 +8191,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -7609,7 +8218,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -7637,7 +8245,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -7665,7 +8272,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -7757,7 +8363,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -7785,7 +8390,6 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
-      <c r="F115" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:F115"/>
@@ -7797,7 +8401,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8490,7 +9094,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -9054,339 +9658,6 @@
     </row>
   </sheetData>
   <autoFilter ref="A4:H16"/>
-  <mergeCells count="3">
-    <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A1:H1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
-    <col width="70" customWidth="1" min="8" max="8"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Club Providencia (000031)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>6 usuario(s) · 2 punto(s) activo(s) · 0 CPA · 2 solo monitoreo</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="28" customHeight="1">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>CPA: —  |  Solo monitoreo: 000031-01, 000031-02</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Email</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Nombre</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Cuenta de esta empresa</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Empresa de la cuenta</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Switch on/off</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Puntos con acceso</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>Node IDs</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>Puntos (nombre)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>fsanchez@clubprovidencia.cl</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>Francisco Sanchez</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>Club Providencia</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>000031-01, 000031-02</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>000031-01 (Matriz Fitness); 000031-02 (Matriz Piscina)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>jarenas@clubprovidencia.cl</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>Abimael Arenas</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>Club Providencia</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>000031-01, 000031-02</t>
-        </is>
-      </c>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>000031-01 (Matriz Fitness); 000031-02 (Matriz Piscina)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>mcastillo@clubprovidencia.cl</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Maikol Castillo</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>Club Providencia</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>000031-01, 000031-02</t>
-        </is>
-      </c>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>000031-01 (Matriz Fitness); 000031-02 (Matriz Piscina)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>osuarez@clubprovidencia.cl</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Omar Suarez</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Club Providencia</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="G8" s="5" t="inlineStr">
-        <is>
-          <t>000031-01, 000031-02</t>
-        </is>
-      </c>
-      <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>000031-01 (Matriz Fitness); 000031-02 (Matriz Piscina)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>fcuevas@expensereduction.com</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Felipe Cuevas</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>Wes Spa</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>000031-01, 000031-02</t>
-        </is>
-      </c>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>000031-01 (Matriz Fitness); 000031-02 (Matriz Piscina)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>go.salass@gmail.com</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Gonzalo Salas</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>Wes Spa</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>000031-01, 000031-02</t>
-        </is>
-      </c>
-      <c r="H10" s="5" t="inlineStr">
-        <is>
-          <t>000031-01 (Matriz Fitness); 000031-02 (Matriz Piscina)</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A4:H10"/>
   <mergeCells count="3">
     <mergeCell ref="A3:H3"/>
     <mergeCell ref="A2:H2"/>
@@ -9418,21 +9689,21 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>COPEC (000009)</t>
+          <t>Club Providencia (000031)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>6 usuario(s) · 11 punto(s) activo(s) · 0 CPA · 11 solo monitoreo</t>
+          <t>6 usuario(s) · 2 punto(s) activo(s) · 0 CPA · 2 solo monitoreo</t>
         </is>
       </c>
     </row>
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>CPA: —  |  Solo monitoreo: 000009-00, 000009-01, 000009-02, 000009-03, 000009-04, 000009-05, 000009-06, 000009-08, 000009-09, 000009-10, 000009-11</t>
+          <t>CPA: —  |  Solo monitoreo: 000031-01, 000031-02</t>
         </is>
       </c>
     </row>
@@ -9481,12 +9752,12 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>60079@escopec.cl</t>
+          <t>fsanchez@clubprovidencia.cl</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Hernan Concesionario</t>
+          <t>Francisco Sanchez</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -9496,7 +9767,7 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>COPEC</t>
+          <t>Club Providencia</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -9505,28 +9776,28 @@
         </is>
       </c>
       <c r="F5" s="5" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>000009-00, 000009-01, 000009-02, 000009-03, 000009-04, 000009-05, 000009-06, 000009-08, 000009-09, 000009-10, 000009-11</t>
+          <t>000031-01, 000031-02</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>000009-00 (Copec Costanera); 000009-01 (Oficina Admin.); 000009-02 (Estanque Reutilización); 000009-03 (Lavado Automático Norte); 000009-04 (Lavado Automático Sur); 000009-05 (Copec Riego); 000009-06 (Copec Matriz Principal); 000009-08 (Copec Pronto Baños); 000009-09 (Copec Lavado Auto servicio Norte); 000009-10 (Copec Lavado Auto servicio Sur); 000009-11 (Copec Pronto Tienda)</t>
+          <t>000031-01 (Matriz Fitness); 000031-02 (Matriz Piscina)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>bivergara@copec.cl</t>
+          <t>jarenas@clubprovidencia.cl</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Benjamin vergara</t>
+          <t>Abimael Arenas</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -9536,7 +9807,7 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>COPEC</t>
+          <t>Club Providencia</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -9545,28 +9816,28 @@
         </is>
       </c>
       <c r="F6" s="5" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>000009-00, 000009-01, 000009-02, 000009-03, 000009-04, 000009-05, 000009-06, 000009-08, 000009-09, 000009-10, 000009-11</t>
+          <t>000031-01, 000031-02</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>000009-00 (Copec Costanera); 000009-01 (Oficina Admin.); 000009-02 (Estanque Reutilización); 000009-03 (Lavado Automático Norte); 000009-04 (Lavado Automático Sur); 000009-05 (Copec Riego); 000009-06 (Copec Matriz Principal); 000009-08 (Copec Pronto Baños); 000009-09 (Copec Lavado Auto servicio Norte); 000009-10 (Copec Lavado Auto servicio Sur); 000009-11 (Copec Pronto Tienda)</t>
+          <t>000031-01 (Matriz Fitness); 000031-02 (Matriz Piscina)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>cagutierrez@copec.cl</t>
+          <t>mcastillo@clubprovidencia.cl</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Cristian Gutierrez</t>
+          <t>Maikol Castillo</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -9576,37 +9847,37 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>COPEC</t>
+          <t>Club Providencia</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="F7" s="5" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>000009-00, 000009-01, 000009-02, 000009-03, 000009-04, 000009-05, 000009-06, 000009-08, 000009-09, 000009-10, 000009-11</t>
+          <t>000031-01, 000031-02</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>000009-00 (Copec Costanera); 000009-01 (Oficina Admin.); 000009-02 (Estanque Reutilización); 000009-03 (Lavado Automático Norte); 000009-04 (Lavado Automático Sur); 000009-05 (Copec Riego); 000009-06 (Copec Matriz Principal); 000009-08 (Copec Pronto Baños); 000009-09 (Copec Lavado Auto servicio Norte); 000009-10 (Copec Lavado Auto servicio Sur); 000009-11 (Copec Pronto Tienda)</t>
+          <t>000031-01 (Matriz Fitness); 000031-02 (Matriz Piscina)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>pronto.costanerae0@arcoprime.cl</t>
+          <t>osuarez@clubprovidencia.cl</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Ximena Puing</t>
+          <t>Omar Suarez</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -9616,7 +9887,7 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>COPEC</t>
+          <t>Club Providencia</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -9625,38 +9896,38 @@
         </is>
       </c>
       <c r="F8" s="5" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>000009-00, 000009-01, 000009-02, 000009-03, 000009-04, 000009-05, 000009-06, 000009-08, 000009-09, 000009-10, 000009-11</t>
+          <t>000031-01, 000031-02</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>000009-00 (Copec Costanera); 000009-01 (Oficina Admin.); 000009-02 (Estanque Reutilización); 000009-03 (Lavado Automático Norte); 000009-04 (Lavado Automático Sur); 000009-05 (Copec Riego); 000009-06 (Copec Matriz Principal); 000009-08 (Copec Pronto Baños); 000009-09 (Copec Lavado Auto servicio Norte); 000009-10 (Copec Lavado Auto servicio Sur); 000009-11 (Copec Pronto Tienda)</t>
+          <t>000031-01 (Matriz Fitness); 000031-02 (Matriz Piscina)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>raosses@fitgal.cl</t>
+          <t>fcuevas@expensereduction.com</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Rene Osses</t>
+          <t>Felipe Cuevas</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>COPEC</t>
+          <t>Wes Spa</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -9665,16 +9936,16 @@
         </is>
       </c>
       <c r="F9" s="5" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>000009-00, 000009-01, 000009-02, 000009-03, 000009-04, 000009-05, 000009-06, 000009-08, 000009-09, 000009-10, 000009-11</t>
+          <t>000031-01, 000031-02</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>000009-00 (Copec Costanera); 000009-01 (Oficina Admin.); 000009-02 (Estanque Reutilización); 000009-03 (Lavado Automático Norte); 000009-04 (Lavado Automático Sur); 000009-05 (Copec Riego); 000009-06 (Copec Matriz Principal); 000009-08 (Copec Pronto Baños); 000009-09 (Copec Lavado Auto servicio Norte); 000009-10 (Copec Lavado Auto servicio Sur); 000009-11 (Copec Pronto Tienda)</t>
+          <t>000031-01 (Matriz Fitness); 000031-02 (Matriz Piscina)</t>
         </is>
       </c>
     </row>
@@ -9705,16 +9976,16 @@
         </is>
       </c>
       <c r="F10" s="5" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>000009-00, 000009-01, 000009-02, 000009-03, 000009-04, 000009-05, 000009-06, 000009-08, 000009-09, 000009-10, 000009-11</t>
+          <t>000031-01, 000031-02</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>000009-00 (Copec Costanera); 000009-01 (Oficina Admin.); 000009-02 (Estanque Reutilización); 000009-03 (Lavado Automático Norte); 000009-04 (Lavado Automático Sur); 000009-05 (Copec Riego); 000009-06 (Copec Matriz Principal); 000009-08 (Copec Pronto Baños); 000009-09 (Copec Lavado Auto servicio Norte); 000009-10 (Copec Lavado Auto servicio Sur); 000009-11 (Copec Pronto Tienda)</t>
+          <t>000031-01 (Matriz Fitness); 000031-02 (Matriz Piscina)</t>
         </is>
       </c>
     </row>
@@ -9730,6 +10001,339 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="70" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>COPEC (000009)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>6 usuario(s) · 11 punto(s) activo(s) · 0 CPA · 11 solo monitoreo</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>CPA: —  |  Solo monitoreo: 000009-00, 000009-01, 000009-02, 000009-03, 000009-04, 000009-05, 000009-06, 000009-08, 000009-09, 000009-10, 000009-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Nombre</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Cuenta de esta empresa</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Empresa de la cuenta</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Switch on/off</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Puntos con acceso</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Node IDs</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Puntos (nombre)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>60079@escopec.cl</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Hernan Concesionario</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>COPEC</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>000009-00, 000009-01, 000009-02, 000009-03, 000009-04, 000009-05, 000009-06, 000009-08, 000009-09, 000009-10, 000009-11</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>000009-00 (Copec Costanera); 000009-01 (Oficina Admin.); 000009-02 (Estanque Reutilización); 000009-03 (Lavado Automático Norte); 000009-04 (Lavado Automático Sur); 000009-05 (Copec Riego); 000009-06 (Copec Matriz Principal); 000009-08 (Copec Pronto Baños); 000009-09 (Copec Lavado Auto servicio Norte); 000009-10 (Copec Lavado Auto servicio Sur); 000009-11 (Copec Pronto Tienda)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>bivergara@copec.cl</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Benjamin vergara</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>COPEC</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>000009-00, 000009-01, 000009-02, 000009-03, 000009-04, 000009-05, 000009-06, 000009-08, 000009-09, 000009-10, 000009-11</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>000009-00 (Copec Costanera); 000009-01 (Oficina Admin.); 000009-02 (Estanque Reutilización); 000009-03 (Lavado Automático Norte); 000009-04 (Lavado Automático Sur); 000009-05 (Copec Riego); 000009-06 (Copec Matriz Principal); 000009-08 (Copec Pronto Baños); 000009-09 (Copec Lavado Auto servicio Norte); 000009-10 (Copec Lavado Auto servicio Sur); 000009-11 (Copec Pronto Tienda)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>cagutierrez@copec.cl</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Cristian Gutierrez</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>COPEC</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>000009-00, 000009-01, 000009-02, 000009-03, 000009-04, 000009-05, 000009-06, 000009-08, 000009-09, 000009-10, 000009-11</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>000009-00 (Copec Costanera); 000009-01 (Oficina Admin.); 000009-02 (Estanque Reutilización); 000009-03 (Lavado Automático Norte); 000009-04 (Lavado Automático Sur); 000009-05 (Copec Riego); 000009-06 (Copec Matriz Principal); 000009-08 (Copec Pronto Baños); 000009-09 (Copec Lavado Auto servicio Norte); 000009-10 (Copec Lavado Auto servicio Sur); 000009-11 (Copec Pronto Tienda)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>pronto.costanerae0@arcoprime.cl</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Ximena Puing</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>COPEC</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>000009-00, 000009-01, 000009-02, 000009-03, 000009-04, 000009-05, 000009-06, 000009-08, 000009-09, 000009-10, 000009-11</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>000009-00 (Copec Costanera); 000009-01 (Oficina Admin.); 000009-02 (Estanque Reutilización); 000009-03 (Lavado Automático Norte); 000009-04 (Lavado Automático Sur); 000009-05 (Copec Riego); 000009-06 (Copec Matriz Principal); 000009-08 (Copec Pronto Baños); 000009-09 (Copec Lavado Auto servicio Norte); 000009-10 (Copec Lavado Auto servicio Sur); 000009-11 (Copec Pronto Tienda)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>raosses@fitgal.cl</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Rene Osses</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>COPEC</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>000009-00, 000009-01, 000009-02, 000009-03, 000009-04, 000009-05, 000009-06, 000009-08, 000009-09, 000009-10, 000009-11</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>000009-00 (Copec Costanera); 000009-01 (Oficina Admin.); 000009-02 (Estanque Reutilización); 000009-03 (Lavado Automático Norte); 000009-04 (Lavado Automático Sur); 000009-05 (Copec Riego); 000009-06 (Copec Matriz Principal); 000009-08 (Copec Pronto Baños); 000009-09 (Copec Lavado Auto servicio Norte); 000009-10 (Copec Lavado Auto servicio Sur); 000009-11 (Copec Pronto Tienda)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>go.salass@gmail.com</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Gonzalo Salas</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Wes Spa</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>000009-00, 000009-01, 000009-02, 000009-03, 000009-04, 000009-05, 000009-06, 000009-08, 000009-09, 000009-10, 000009-11</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>000009-00 (Copec Costanera); 000009-01 (Oficina Admin.); 000009-02 (Estanque Reutilización); 000009-03 (Lavado Automático Norte); 000009-04 (Lavado Automático Sur); 000009-05 (Copec Riego); 000009-06 (Copec Matriz Principal); 000009-08 (Copec Pronto Baños); 000009-09 (Copec Lavado Auto servicio Norte); 000009-10 (Copec Lavado Auto servicio Sur); 000009-11 (Copec Pronto Tienda)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:H10"/>
+  <mergeCells count="3">
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -9893,139 +10497,6 @@
     </row>
   </sheetData>
   <autoFilter ref="A4:H6"/>
-  <mergeCells count="3">
-    <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A1:H1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
-    <col width="70" customWidth="1" min="8" max="8"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Corporación Puente Alto (000010)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>1 usuario(s) · 11 punto(s) activo(s) · 0 CPA · 11 solo monitoreo</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="28" customHeight="1">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>CPA: —  |  Solo monitoreo: 000010-01, 000010-02, 000010-03, 000010-04, 000010-05, 000010-06, 000010-07, 000010-08, 000010-09, 000010-10, 000010-11</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Email</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Nombre</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Cuenta de esta empresa</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Empresa de la cuenta</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Switch on/off</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Puntos con acceso</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>Node IDs</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>Puntos (nombre)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>go.salass@gmail.com</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>Gonzalo Salas</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>Wes Spa</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="n">
-        <v>11</v>
-      </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>000010-01, 000010-02, 000010-03, 000010-04, 000010-05, 000010-06, 000010-07, 000010-08, 000010-09, 000010-10, 000010-11</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>000010-01 (Escuela Andes del SUR); 000010-02 (Esc. Villa Independencia); 000010-03 (Esc. Padre Hurtado); 000010-04 (Colegio Maipo); 000010-05 (Esc. Luis Matte Larraín); 000010-06 (Esc. Gabriela); 000010-07 (Esc. Juan Mackenna); 000010-08 (Liceo Chiloé); 000010-09 (Esc. Los Andes); 000010-10 (Consolidada); 000010-11 (Esc. Nonato Coo)</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A4:H5"/>
   <mergeCells count="3">
     <mergeCell ref="A3:H3"/>
     <mergeCell ref="A2:H2"/>
@@ -10057,21 +10528,21 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>DERCO (000012)</t>
+          <t>Corporación Puente Alto (000010)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1 usuario(s) · 7 punto(s) activo(s) · 0 CPA · 7 solo monitoreo</t>
+          <t>1 usuario(s) · 11 punto(s) activo(s) · 0 CPA · 11 solo monitoreo</t>
         </is>
       </c>
     </row>
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>CPA: —  |  Solo monitoreo: 000012-06, 000012-07, 000012-08, 000012-09, 000012-10, 000012-11, 000012-12</t>
+          <t>CPA: —  |  Solo monitoreo: 000010-01, 000010-02, 000010-03, 000010-04, 000010-05, 000010-06, 000010-07, 000010-08, 000010-09, 000010-10, 000010-11</t>
         </is>
       </c>
     </row>
@@ -10144,16 +10615,16 @@
         </is>
       </c>
       <c r="F5" s="5" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>000012-06, 000012-07, 000012-08, 000012-09, 000012-10, 000012-11, 000012-12</t>
+          <t>000010-01, 000010-02, 000010-03, 000010-04, 000010-05, 000010-06, 000010-07, 000010-08, 000010-09, 000010-10, 000010-11</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>000012-06 (Quilicura Matriz Principal); 000012-07 (Quilicura Dercomaq); 000012-08 (Quilicura Lav. de Maquinas); 000012-09 (Quilicura Casino); 000012-10 (Quilicura Proderco); 000012-11 (Quilicura Camarines); 000012-12 (Quilicura Edificio JCB)</t>
+          <t>000010-01 (Escuela Andes del SUR); 000010-02 (Esc. Villa Independencia); 000010-03 (Esc. Padre Hurtado); 000010-04 (Colegio Maipo); 000010-05 (Esc. Luis Matte Larraín); 000010-06 (Esc. Gabriela); 000010-07 (Esc. Juan Mackenna); 000010-08 (Liceo Chiloé); 000010-09 (Esc. Los Andes); 000010-10 (Consolidada); 000010-11 (Esc. Nonato Coo)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Corregir mapeo CPA: leer todo el Excel de horarios
El parser cortaba en la columna L y se perdían colegios CORMUP y
los puntos de Renca. Ahora CORMUP queda 11/14 CPA y Renca 5/5.

Co-authored-by: anibaloperacionesWes <anibaloperacionesWes@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/Usuarios/acceso_por_empresa/accesos_por_empresa.xlsx
+++ b/reports/Usuarios/acceso_por_empresa/accesos_por_empresa.xlsx
@@ -30,7 +30,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$4:$I$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CPA control'!$A$4:$F$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CPA control'!$A$4:$F$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Puntos'!$A$4:$F$115</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'000020 AGUNSA'!$A$4:$H$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'000021 CDUC'!$A$4:$H$16</definedName>
@@ -734,22 +734,22 @@
         <v>14</v>
       </c>
       <c r="D9" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="E9" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="F9" t="n">
         <v>2</v>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>000008-01, 000008-03, 000008-04, 000008-05</t>
+          <t>000008-01, 000008-03, 000008-04, 000008-05, 000008-06, 000008-07, 000008-09, 000008-10, 000008-11, 000008-12, 000008-14</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>000008-02, 000008-06, 000008-07, 000008-08, 000008-09, 000008-10, 000008-11, 000008-12, 000008-13, 000008-14</t>
+          <t>000008-02, 000008-08, 000008-13</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -808,18 +808,22 @@
         <v>7</v>
       </c>
       <c r="D11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F11" t="n">
         <v>1</v>
       </c>
-      <c r="G11" s="5" t="inlineStr"/>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>000012-06</t>
+        </is>
+      </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>000012-06, 000012-07, 000012-08, 000012-09, 000012-10, 000012-11, 000012-12</t>
+          <t>000012-07, 000012-08, 000012-09, 000012-10, 000012-11, 000012-12</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -948,20 +952,20 @@
         <v>1</v>
       </c>
       <c r="D15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" t="n">
         <v>0</v>
-      </c>
-      <c r="E15" t="n">
-        <v>1</v>
       </c>
       <c r="F15" t="n">
         <v>1</v>
       </c>
-      <c r="G15" s="5" t="inlineStr"/>
-      <c r="H15" s="5" t="inlineStr">
+      <c r="G15" s="5" t="inlineStr">
         <is>
           <t>000022-00</t>
         </is>
       </c>
+      <c r="H15" s="5" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
           <t>000022 Las Condes</t>
@@ -1057,22 +1061,22 @@
         <v>25</v>
       </c>
       <c r="D18" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E18" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F18" t="n">
         <v>25</v>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>000025-01, 000025-07, 000025-19</t>
+          <t>000025-01, 000025-07, 000025-18, 000025-19</t>
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>000025-04, 000025-08, 000025-10, 000025-12, 000025-13, 000025-17, 000025-18, 000025-20, 000025-21, 000025-22, 000025-23, 000025-24, 000025-27, 000025-28, 000025-29, 000025-32, 000025-33, 000025-34, 000025-35, 000025-36, 000025-37, 000025-38</t>
+          <t>000025-04, 000025-08, 000025-10, 000025-12, 000025-13, 000025-17, 000025-20, 000025-21, 000025-22, 000025-23, 000025-24, 000025-27, 000025-28, 000025-29, 000025-32, 000025-33, 000025-34, 000025-35, 000025-36, 000025-37, 000025-38</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1096,20 +1100,20 @@
         <v>4</v>
       </c>
       <c r="D19" t="n">
+        <v>4</v>
+      </c>
+      <c r="E19" t="n">
         <v>0</v>
-      </c>
-      <c r="E19" t="n">
-        <v>4</v>
       </c>
       <c r="F19" t="n">
         <v>12</v>
       </c>
-      <c r="G19" s="5" t="inlineStr"/>
-      <c r="H19" s="5" t="inlineStr">
+      <c r="G19" s="5" t="inlineStr">
         <is>
           <t>000006-01, 000006-02, 000006-04, 000006-05</t>
         </is>
       </c>
+      <c r="H19" s="5" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
           <t>000006 Providencia</t>
@@ -1131,24 +1135,20 @@
         <v>5</v>
       </c>
       <c r="D20" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F20" t="n">
         <v>1</v>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>000017-07, 000017-08</t>
-        </is>
-      </c>
-      <c r="H20" s="5" t="inlineStr">
-        <is>
-          <t>000017-04, 000017-05, 000017-06</t>
-        </is>
-      </c>
+          <t>000017-04, 000017-05, 000017-06, 000017-07, 000017-08</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
           <t>000017 Renca</t>
@@ -1229,14 +1229,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1 usuario(s) · 7 punto(s) activo(s) · 0 CPA · 7 solo monitoreo</t>
+          <t>1 usuario(s) · 7 punto(s) activo(s) · 1 CPA · 6 solo monitoreo</t>
         </is>
       </c>
     </row>
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>CPA: —  |  Solo monitoreo: 000012-06, 000012-07, 000012-08, 000012-09, 000012-10, 000012-11, 000012-12</t>
+          <t>CPA: 000012-06  |  Solo monitoreo: 000012-07, 000012-08, 000012-09, 000012-10, 000012-11, 000012-12</t>
         </is>
       </c>
     </row>
@@ -2041,14 +2041,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1 usuario(s) · 1 punto(s) activo(s) · 0 CPA · 1 solo monitoreo</t>
+          <t>1 usuario(s) · 1 punto(s) activo(s) · 1 CPA · 0 solo monitoreo</t>
         </is>
       </c>
     </row>
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>CPA: —  |  Solo monitoreo: 000022-00</t>
+          <t>CPA: 000022-00  |  Solo monitoreo: —</t>
         </is>
       </c>
     </row>
@@ -2760,14 +2760,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>25 usuario(s) · 25 punto(s) activo(s) · 3 CPA · 22 solo monitoreo</t>
+          <t>25 usuario(s) · 25 punto(s) activo(s) · 4 CPA · 21 solo monitoreo</t>
         </is>
       </c>
     </row>
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>CPA: 000025-01, 000025-07, 000025-19  |  Solo monitoreo: 000025-04, 000025-08, 000025-10, 000025-12, 000025-13, 000025-17, 000025-18, 000025-20, 000025-21, 000025-22, 000025-23, 000025-24, 000025-27, 000025-28, 000025-29, 000025-32, 000025-33, 000025-34, 000025-35, 000025-36, 000025-37, 000025-38</t>
+          <t>CPA: 000025-01, 000025-07, 000025-18, 000025-19  |  Solo monitoreo: 000025-04, 000025-08, 000025-10, 000025-12, 000025-13, 000025-17, 000025-20, 000025-21, 000025-22, 000025-23, 000025-24, 000025-27, 000025-28, 000025-29, 000025-32, 000025-33, 000025-34, 000025-35, 000025-36, 000025-37, 000025-38</t>
         </is>
       </c>
     </row>
@@ -3853,14 +3853,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>12 usuario(s) · 4 punto(s) activo(s) · 0 CPA · 4 solo monitoreo</t>
+          <t>12 usuario(s) · 4 punto(s) activo(s) · 4 CPA · 0 solo monitoreo</t>
         </is>
       </c>
     </row>
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>CPA: —  |  Solo monitoreo: 000006-01, 000006-02, 000006-04, 000006-05</t>
+          <t>CPA: 000006-01, 000006-02, 000006-04, 000006-05  |  Solo monitoreo: —</t>
         </is>
       </c>
     </row>
@@ -4426,14 +4426,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1 usuario(s) · 5 punto(s) activo(s) · 2 CPA · 3 solo monitoreo</t>
+          <t>1 usuario(s) · 5 punto(s) activo(s) · 5 CPA · 0 solo monitoreo</t>
         </is>
       </c>
     </row>
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>CPA: 000017-07, 000017-08  |  Solo monitoreo: 000017-04, 000017-05, 000017-06</t>
+          <t>CPA: 000017-04, 000017-05, 000017-06, 000017-07, 000017-08  |  Solo monitoreo: —</t>
         </is>
       </c>
     </row>
@@ -4536,7 +4536,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4820,22 +4820,22 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>000028-01</t>
+          <t>000008-06</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Liceo Alto Cordillera</t>
+          <t>Luis Arrieta Caña</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>000028</t>
+          <t>000008</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>La Florida</t>
+          <t>CORMUP</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -4845,29 +4845,29 @@
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>liceo alto cordillera la florida</t>
+          <t>luis arrieta cañas</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>000024-01</t>
+          <t>000008-07</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Eugenio María De Hostos</t>
+          <t>Erasmo Escala</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>000024</t>
+          <t>000008</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>La Reina</t>
+          <t>CORMUP</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
@@ -4877,29 +4877,29 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>eugenio maria de hostos</t>
+          <t>Colegio erasmo escala</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>000002-01</t>
+          <t>000008-09</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Lo Valledor - P1</t>
+          <t>Juan Bautista Pasten</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>000002</t>
+          <t>000008</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Lo valledor</t>
+          <t>CORMUP</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
@@ -4909,29 +4909,29 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>lo valledor p1</t>
+          <t>juan bautista pastene</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>000025-01</t>
+          <t>000008-10</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Estanque Norte Locales Mall</t>
+          <t>Matilde Huici Navas</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>000025</t>
+          <t>000008</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Parque Arauco</t>
+          <t>CORMUP</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
@@ -4941,29 +4941,29 @@
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>PAE estanquer norte locales</t>
+          <t>matilde huichinavas</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>000025-07</t>
+          <t>000008-11</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>PIZZA HUT</t>
+          <t>CE Valle Hermoso</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>000025</t>
+          <t>000008</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Parque Arauco</t>
+          <t>CORMUP</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
@@ -4973,29 +4973,29 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>pizza hut</t>
+          <t>ce valle germoso</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>000025-19</t>
+          <t>000008-12</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Sala de Bomba Estanque Sur</t>
+          <t>Unión Nacional Árabe</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>000025</t>
+          <t>000008</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Parque Arauco</t>
+          <t>CORMUP</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
@@ -5005,29 +5005,29 @@
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>mae  sala de bomba estanque sur</t>
+          <t>union nacional arabe</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>000017-07</t>
+          <t>000008-14</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Cumbre de cóndores pte.</t>
+          <t>Juan Pablo II</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>000017</t>
+          <t>000008</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Renca</t>
+          <t>CORMUP</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
@@ -5037,44 +5037,588 @@
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>ICCP</t>
+          <t>juan pablo segundo</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
+          <t>000012-06</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Quilicura Matriz Principal</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>000012</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>DERCO</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>CPA (monitoreo con control)</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Derco matriz principal</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>000028-01</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Liceo Alto Cordillera</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>000028</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>La Florida</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>CPA (monitoreo con control)</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>liceo alto cordillera la florida</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>000024-01</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Eugenio María De Hostos</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>000024</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>La Reina</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>CPA (monitoreo con control)</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>eugenio maria de hostos</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>000022-00</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Alexander Fleming</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>000022</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Las Condes</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>CPA (monitoreo con control)</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>escuela alexander fleming</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>000002-01</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Lo Valledor - P1</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>000002</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>Lo valledor</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>CPA (monitoreo con control)</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>lo valledor p1</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>000025-01</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Estanque Norte Locales Mall</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>000025</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>Parque Arauco</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>CPA (monitoreo con control)</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>PAE estanquer norte locales</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>000025-07</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>PIZZA HUT</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>000025</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>Parque Arauco</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>CPA (monitoreo con control)</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>pizza hut</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>000025-18</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>San Ignacio 500</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>000025</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>Parque Arauco</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>CPA (monitoreo con control)</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>san ignacio 500</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>000025-19</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Sala de Bomba Estanque Sur</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>000025</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>Parque Arauco</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>CPA (monitoreo con control)</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>mae  sala de bomba estanque sur</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>000006-01</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Liceo Lastarria</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>000006</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>Providencia</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>CPA (monitoreo con control)</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>las tarrias providencia</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>000006-02</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Carmela Carvajal</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>000006</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>Providencia</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>CPA (monitoreo con control)</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>carmela carvajal provi</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>000006-04</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Liceo 7 Luisa Saavedra</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>000006</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>Providencia</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>CPA (monitoreo con control)</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>liceo 7 luisa saavedra</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>000006-05</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Liceo Juan Pablo Duarte</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>000006</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>Providencia</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>CPA (monitoreo con control)</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>liceo juan pablo duarte</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>000017-04</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Esc. Lo Velásquez</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>000017</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>Renca</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>CPA (monitoreo con control)</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>escuela lo velazques</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>000017-05</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Gimnasio</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>000017</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>Renca</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>CPA (monitoreo con control)</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>GYM renca</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>000017-06</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Piscina Municipal</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>000017</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>Renca</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>CPA (monitoreo con control)</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>Picina municipal renca</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>000017-07</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Cumbre de cóndores pte.</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>000017</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>Renca</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>CPA (monitoreo con control)</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>ICCP</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
           <t>000017-08</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B36" s="3" t="inlineStr">
         <is>
           <t>Cumbre de cóndores Ote.</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="C36" s="3" t="inlineStr">
         <is>
           <t>000017</t>
         </is>
       </c>
-      <c r="D19" s="3" t="inlineStr">
+      <c r="D36" s="3" t="inlineStr">
         <is>
           <t>Renca</t>
         </is>
       </c>
-      <c r="E19" s="3" t="inlineStr">
+      <c r="E36" s="3" t="inlineStr">
         <is>
           <t>CPA (monitoreo con control)</t>
         </is>
       </c>
-      <c r="F19" s="3" t="inlineStr">
+      <c r="F36" s="3" t="inlineStr">
         <is>
           <t>ICCO</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:F19"/>
+  <autoFilter ref="A4:F36"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
@@ -5345,6 +5889,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -5404,6 +5949,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -5431,6 +5977,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -5458,6 +6005,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -5549,6 +6097,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -5576,6 +6125,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -5603,6 +6153,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -5630,6 +6181,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -5657,6 +6209,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -5684,6 +6237,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -5711,6 +6265,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -5738,6 +6293,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -5765,6 +6321,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -5792,6 +6349,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -5819,6 +6377,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -5846,6 +6405,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -5873,6 +6433,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -5900,6 +6461,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -5927,6 +6489,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -5954,6 +6517,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -6013,6 +6577,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -6131,9 +6696,14 @@
           <t>CORMUP</t>
         </is>
       </c>
-      <c r="E33" s="4" t="inlineStr">
-        <is>
-          <t>Solo monitoreo</t>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>CPA (monitoreo con control)</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>luis arrieta cañas</t>
         </is>
       </c>
     </row>
@@ -6158,9 +6728,14 @@
           <t>CORMUP</t>
         </is>
       </c>
-      <c r="E34" s="4" t="inlineStr">
-        <is>
-          <t>Solo monitoreo</t>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>CPA (monitoreo con control)</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Colegio erasmo escala</t>
         </is>
       </c>
     </row>
@@ -6190,6 +6765,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -6212,9 +6788,14 @@
           <t>CORMUP</t>
         </is>
       </c>
-      <c r="E36" s="4" t="inlineStr">
-        <is>
-          <t>Solo monitoreo</t>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>CPA (monitoreo con control)</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>juan bautista pastene</t>
         </is>
       </c>
     </row>
@@ -6239,9 +6820,14 @@
           <t>CORMUP</t>
         </is>
       </c>
-      <c r="E37" s="4" t="inlineStr">
-        <is>
-          <t>Solo monitoreo</t>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>CPA (monitoreo con control)</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>matilde huichinavas</t>
         </is>
       </c>
     </row>
@@ -6266,9 +6852,14 @@
           <t>CORMUP</t>
         </is>
       </c>
-      <c r="E38" s="4" t="inlineStr">
-        <is>
-          <t>Solo monitoreo</t>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>CPA (monitoreo con control)</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>ce valle germoso</t>
         </is>
       </c>
     </row>
@@ -6293,9 +6884,14 @@
           <t>CORMUP</t>
         </is>
       </c>
-      <c r="E39" s="4" t="inlineStr">
-        <is>
-          <t>Solo monitoreo</t>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>CPA (monitoreo con control)</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>union nacional arabe</t>
         </is>
       </c>
     </row>
@@ -6325,6 +6921,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -6347,9 +6944,14 @@
           <t>CORMUP</t>
         </is>
       </c>
-      <c r="E41" s="4" t="inlineStr">
-        <is>
-          <t>Solo monitoreo</t>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>CPA (monitoreo con control)</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>juan pablo segundo</t>
         </is>
       </c>
     </row>
@@ -6379,6 +6981,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -6406,6 +7009,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -6433,6 +7037,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -6460,6 +7065,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -6487,6 +7093,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -6514,6 +7121,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -6541,6 +7149,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -6568,6 +7177,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -6595,6 +7205,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -6622,6 +7233,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -6649,6 +7261,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -6671,9 +7284,14 @@
           <t>DERCO</t>
         </is>
       </c>
-      <c r="E53" s="4" t="inlineStr">
-        <is>
-          <t>Solo monitoreo</t>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>CPA (monitoreo con control)</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Derco matriz principal</t>
         </is>
       </c>
     </row>
@@ -6703,6 +7321,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -6730,6 +7349,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -6757,6 +7377,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -6784,6 +7405,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -6811,6 +7433,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -6838,6 +7461,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -6865,6 +7489,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -6892,6 +7517,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -6919,6 +7545,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -6946,6 +7573,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -6973,6 +7601,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -7000,6 +7629,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -7027,6 +7657,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -7054,6 +7685,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -7140,9 +7772,14 @@
           <t>Las Condes</t>
         </is>
       </c>
-      <c r="E70" s="4" t="inlineStr">
-        <is>
-          <t>Solo monitoreo</t>
+      <c r="E70" s="3" t="inlineStr">
+        <is>
+          <t>CPA (monitoreo con control)</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>escuela alexander fleming</t>
         </is>
       </c>
     </row>
@@ -7204,6 +7841,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -7231,6 +7869,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -7258,6 +7897,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -7285,6 +7925,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -7312,6 +7953,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -7339,6 +7981,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -7366,6 +8009,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -7393,6 +8037,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -7452,6 +8097,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -7511,6 +8157,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -7538,6 +8185,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -7565,6 +8213,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -7592,6 +8241,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -7619,6 +8269,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -7641,9 +8292,14 @@
           <t>Parque Arauco</t>
         </is>
       </c>
-      <c r="E88" s="4" t="inlineStr">
-        <is>
-          <t>Solo monitoreo</t>
+      <c r="E88" s="3" t="inlineStr">
+        <is>
+          <t>CPA (monitoreo con control)</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>san ignacio 500</t>
         </is>
       </c>
     </row>
@@ -7705,6 +8361,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -7732,6 +8389,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -7759,6 +8417,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -7786,6 +8445,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -7813,6 +8473,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -7840,6 +8501,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -7867,6 +8529,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -7894,6 +8557,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -7921,6 +8585,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -7948,6 +8613,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -7975,6 +8641,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -8002,6 +8669,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -8029,6 +8697,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -8056,6 +8725,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -8083,6 +8753,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -8105,9 +8776,14 @@
           <t>Providencia</t>
         </is>
       </c>
-      <c r="E105" s="4" t="inlineStr">
-        <is>
-          <t>Solo monitoreo</t>
+      <c r="E105" s="3" t="inlineStr">
+        <is>
+          <t>CPA (monitoreo con control)</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>las tarrias providencia</t>
         </is>
       </c>
     </row>
@@ -8132,9 +8808,14 @@
           <t>Providencia</t>
         </is>
       </c>
-      <c r="E106" s="4" t="inlineStr">
-        <is>
-          <t>Solo monitoreo</t>
+      <c r="E106" s="3" t="inlineStr">
+        <is>
+          <t>CPA (monitoreo con control)</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>carmela carvajal provi</t>
         </is>
       </c>
     </row>
@@ -8159,9 +8840,14 @@
           <t>Providencia</t>
         </is>
       </c>
-      <c r="E107" s="4" t="inlineStr">
-        <is>
-          <t>Solo monitoreo</t>
+      <c r="E107" s="3" t="inlineStr">
+        <is>
+          <t>CPA (monitoreo con control)</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>liceo 7 luisa saavedra</t>
         </is>
       </c>
     </row>
@@ -8186,9 +8872,14 @@
           <t>Providencia</t>
         </is>
       </c>
-      <c r="E108" s="4" t="inlineStr">
-        <is>
-          <t>Solo monitoreo</t>
+      <c r="E108" s="3" t="inlineStr">
+        <is>
+          <t>CPA (monitoreo con control)</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>liceo juan pablo duarte</t>
         </is>
       </c>
     </row>
@@ -8213,9 +8904,14 @@
           <t>Renca</t>
         </is>
       </c>
-      <c r="E109" s="4" t="inlineStr">
-        <is>
-          <t>Solo monitoreo</t>
+      <c r="E109" s="3" t="inlineStr">
+        <is>
+          <t>CPA (monitoreo con control)</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>escuela lo velazques</t>
         </is>
       </c>
     </row>
@@ -8240,9 +8936,14 @@
           <t>Renca</t>
         </is>
       </c>
-      <c r="E110" s="4" t="inlineStr">
-        <is>
-          <t>Solo monitoreo</t>
+      <c r="E110" s="3" t="inlineStr">
+        <is>
+          <t>CPA (monitoreo con control)</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>GYM renca</t>
         </is>
       </c>
     </row>
@@ -8267,9 +8968,14 @@
           <t>Renca</t>
         </is>
       </c>
-      <c r="E111" s="4" t="inlineStr">
-        <is>
-          <t>Solo monitoreo</t>
+      <c r="E111" s="3" t="inlineStr">
+        <is>
+          <t>CPA (monitoreo con control)</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>Picina municipal renca</t>
         </is>
       </c>
     </row>
@@ -8363,6 +9069,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -8390,6 +9097,7 @@
           <t>Solo monitoreo</t>
         </is>
       </c>
+      <c r="F115" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:F115"/>
@@ -10362,14 +11070,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2 usuario(s) · 14 punto(s) activo(s) · 4 CPA · 10 solo monitoreo</t>
+          <t>2 usuario(s) · 14 punto(s) activo(s) · 11 CPA · 3 solo monitoreo</t>
         </is>
       </c>
     </row>
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>CPA: 000008-01, 000008-03, 000008-04, 000008-05  |  Solo monitoreo: 000008-02, 000008-06, 000008-07, 000008-08, 000008-09, 000008-10, 000008-11, 000008-12, 000008-13, 000008-14</t>
+          <t>CPA: 000008-01, 000008-03, 000008-04, 000008-05, 000008-06, 000008-07, 000008-09, 000008-10, 000008-11, 000008-12, 000008-14  |  Solo monitoreo: 000008-02, 000008-08, 000008-13</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
PDF: consolidar en una celda los puntos del mismo gabinete
Nueva columna Gabinetes en la hoja 1: si varios nodos comparten gabinete
(listado de equipos vigentes) cuentan como 1 y se listan juntos.

Co-authored-by: anibaloperacionesWes <anibaloperacionesWes@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/Usuarios/acceso_por_empresa/accesos_por_empresa.xlsx
+++ b/reports/Usuarios/acceso_por_empresa/accesos_por_empresa.xlsx
@@ -28,7 +28,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="000026 UDD" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$4:$I$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$4:$K$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CPA control'!$A$4:$F$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Puntos'!$A$4:$F$104</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'000020 AGUNSA'!$A$4:$H$19</definedName>
@@ -494,18 +494,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:K20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="36" customWidth="1" min="7" max="7"/>
-    <col width="42" customWidth="1" min="8" max="8"/>
-    <col width="26" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="36" customWidth="1" min="8" max="8"/>
+    <col width="42" customWidth="1" min="9" max="9"/>
+    <col width="48" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -518,10 +520,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generado 28/08/2026 09:12 hora Chile · se omite personal WES (@wes.cl); se incluye go.salass@gmail.com. CPA = monitoreo con control (horarios programados Drive). Solo monitoreo = punto activo sin CPA.</t>
-        </is>
-      </c>
-    </row>
+          <t>Generado 28/08/2026 09:12 hora Chile · se omite personal WES (@wes.cl); se incluye go.salass@gmail.com. CPA = monitoreo con control (horarios programados Drive). Solo monitoreo = punto activo sin CPA. Gabinetes: puntos en el mismo gabinete cuentan como 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
@@ -540,30 +543,40 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
+          <t>gabinetes</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
           <t>puntos_CPA</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>puntos_solo_monitoreo</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>usuarios_con_acceso</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>ids_CPA</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>ids_solo_monitoreo</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>mismo_gabinete</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>hoja</t>
         </is>
@@ -584,25 +597,33 @@
         <v>5</v>
       </c>
       <c r="D5" t="n">
+        <v>5</v>
+      </c>
+      <c r="E5" t="n">
         <v>1</v>
       </c>
-      <c r="E5" t="n">
+      <c r="F5" t="n">
         <v>4</v>
       </c>
-      <c r="F5" t="n">
+      <c r="G5" t="n">
         <v>15</v>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>000020-02</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="I5" s="5" t="inlineStr">
         <is>
           <t>000020-01, 000020-03, 000020-04, 000020-05</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
         <is>
           <t>000020 AGUNSA</t>
         </is>
@@ -623,25 +644,33 @@
         <v>5</v>
       </c>
       <c r="D6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E6" t="n">
         <v>2</v>
       </c>
-      <c r="E6" t="n">
+      <c r="F6" t="n">
         <v>3</v>
       </c>
-      <c r="F6" t="n">
+      <c r="G6" t="n">
         <v>12</v>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>000021-01, 000021-03</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="I6" s="5" t="inlineStr">
         <is>
           <t>000021-04, 000021-05, 000021-07</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
         <is>
           <t>000021 CDUC</t>
         </is>
@@ -662,21 +691,29 @@
         <v>2</v>
       </c>
       <c r="D7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" t="n">
         <v>0</v>
       </c>
-      <c r="E7" t="n">
+      <c r="F7" t="n">
         <v>2</v>
       </c>
-      <c r="F7" t="n">
+      <c r="G7" t="n">
         <v>6</v>
       </c>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="H7" s="5" t="inlineStr"/>
+      <c r="I7" s="5" t="inlineStr">
         <is>
           <t>000031-01, 000031-02</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
         <is>
           <t>000031 Club Providencia</t>
         </is>
@@ -697,21 +734,29 @@
         <v>11</v>
       </c>
       <c r="D8" t="n">
+        <v>4</v>
+      </c>
+      <c r="E8" t="n">
         <v>0</v>
       </c>
-      <c r="E8" t="n">
+      <c r="F8" t="n">
         <v>11</v>
       </c>
-      <c r="F8" t="n">
+      <c r="G8" t="n">
         <v>6</v>
       </c>
-      <c r="G8" s="5" t="inlineStr"/>
-      <c r="H8" s="5" t="inlineStr">
+      <c r="H8" s="5" t="inlineStr"/>
+      <c r="I8" s="5" t="inlineStr">
         <is>
           <t>000009-00, 000009-01, 000009-02, 000009-03, 000009-04, 000009-05, 000009-06, 000009-08, 000009-09, 000009-10, 000009-11</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>Costanera / Oficina Admin.: 000009-00, 000009-01 · Matriz / riego / estanque: 000009-02, 000009-05, 000009-06 · Lavados: 000009-03, 000009-04, 000009-09, 000009-10 · Pronto: 000009-08, 000009-11</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
         <is>
           <t>000009 COPEC</t>
         </is>
@@ -732,25 +777,33 @@
         <v>14</v>
       </c>
       <c r="D9" t="n">
+        <v>14</v>
+      </c>
+      <c r="E9" t="n">
         <v>11</v>
       </c>
-      <c r="E9" t="n">
+      <c r="F9" t="n">
         <v>3</v>
       </c>
-      <c r="F9" t="n">
+      <c r="G9" t="n">
         <v>2</v>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="H9" s="5" t="inlineStr">
         <is>
           <t>000008-01, 000008-03, 000008-04, 000008-05, 000008-06, 000008-07, 000008-09, 000008-10, 000008-11, 000008-12, 000008-14</t>
         </is>
       </c>
-      <c r="H9" s="5" t="inlineStr">
+      <c r="I9" s="5" t="inlineStr">
         <is>
           <t>000008-02, 000008-08, 000008-13</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
         <is>
           <t>000008 CORMUP</t>
         </is>
@@ -771,25 +824,33 @@
         <v>7</v>
       </c>
       <c r="D10" t="n">
+        <v>7</v>
+      </c>
+      <c r="E10" t="n">
         <v>1</v>
       </c>
-      <c r="E10" t="n">
+      <c r="F10" t="n">
         <v>6</v>
       </c>
-      <c r="F10" t="n">
+      <c r="G10" t="n">
         <v>1</v>
       </c>
-      <c r="G10" s="5" t="inlineStr">
+      <c r="H10" s="5" t="inlineStr">
         <is>
           <t>000012-06</t>
         </is>
       </c>
-      <c r="H10" s="5" t="inlineStr">
+      <c r="I10" s="5" t="inlineStr">
         <is>
           <t>000012-07, 000012-08, 000012-09, 000012-10, 000012-11, 000012-12</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
         <is>
           <t>000012 DERCO</t>
         </is>
@@ -810,21 +871,29 @@
         <v>8</v>
       </c>
       <c r="D11" t="n">
+        <v>7</v>
+      </c>
+      <c r="E11" t="n">
         <v>0</v>
       </c>
-      <c r="E11" t="n">
+      <c r="F11" t="n">
         <v>8</v>
       </c>
-      <c r="F11" t="n">
+      <c r="G11" t="n">
         <v>7</v>
       </c>
-      <c r="G11" s="5" t="inlineStr"/>
-      <c r="H11" s="5" t="inlineStr">
+      <c r="H11" s="5" t="inlineStr"/>
+      <c r="I11" s="5" t="inlineStr">
         <is>
           <t>000027-01, 000027-02, 000027-03, 000027-04, 000027-06, 000027-07, 000027-08, 000027-09</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>Etapa 1-4 y Etapa 5: 000027-03, 000027-04</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
         <is>
           <t>000027 Fundo Zapallar</t>
         </is>
@@ -848,18 +917,26 @@
         <v>1</v>
       </c>
       <c r="E12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" t="n">
         <v>0</v>
       </c>
-      <c r="F12" t="n">
+      <c r="G12" t="n">
         <v>1</v>
       </c>
-      <c r="G12" s="5" t="inlineStr">
+      <c r="H12" s="5" t="inlineStr">
         <is>
           <t>000028-01</t>
         </is>
       </c>
-      <c r="H12" s="5" t="inlineStr"/>
-      <c r="I12" t="inlineStr">
+      <c r="I12" s="5" t="inlineStr"/>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
         <is>
           <t>000028 La Florida</t>
         </is>
@@ -883,18 +960,26 @@
         <v>1</v>
       </c>
       <c r="E13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" t="n">
         <v>0</v>
       </c>
-      <c r="F13" t="n">
+      <c r="G13" t="n">
         <v>2</v>
       </c>
-      <c r="G13" s="5" t="inlineStr">
+      <c r="H13" s="5" t="inlineStr">
         <is>
           <t>000024-01</t>
         </is>
       </c>
-      <c r="H13" s="5" t="inlineStr"/>
-      <c r="I13" t="inlineStr">
+      <c r="I13" s="5" t="inlineStr"/>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
         <is>
           <t>000024 La Reina</t>
         </is>
@@ -918,18 +1003,26 @@
         <v>1</v>
       </c>
       <c r="E14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" t="n">
         <v>0</v>
       </c>
-      <c r="F14" t="n">
+      <c r="G14" t="n">
         <v>1</v>
       </c>
-      <c r="G14" s="5" t="inlineStr">
+      <c r="H14" s="5" t="inlineStr">
         <is>
           <t>000022-00</t>
         </is>
       </c>
-      <c r="H14" s="5" t="inlineStr"/>
-      <c r="I14" t="inlineStr">
+      <c r="I14" s="5" t="inlineStr"/>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
         <is>
           <t>000022 Las Condes</t>
         </is>
@@ -950,25 +1043,33 @@
         <v>2</v>
       </c>
       <c r="D15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E15" t="n">
         <v>1</v>
       </c>
       <c r="F15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" t="n">
         <v>6</v>
       </c>
-      <c r="G15" s="5" t="inlineStr">
+      <c r="H15" s="5" t="inlineStr">
         <is>
           <t>000002-01</t>
         </is>
       </c>
-      <c r="H15" s="5" t="inlineStr">
+      <c r="I15" s="5" t="inlineStr">
         <is>
           <t>000002-03</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
         <is>
           <t>000002 Lo valledor</t>
         </is>
@@ -989,21 +1090,29 @@
         <v>7</v>
       </c>
       <c r="D16" t="n">
+        <v>5</v>
+      </c>
+      <c r="E16" t="n">
         <v>0</v>
       </c>
-      <c r="E16" t="n">
+      <c r="F16" t="n">
         <v>7</v>
       </c>
-      <c r="F16" t="n">
+      <c r="G16" t="n">
         <v>4</v>
       </c>
-      <c r="G16" s="5" t="inlineStr"/>
-      <c r="H16" s="5" t="inlineStr">
+      <c r="H16" s="5" t="inlineStr"/>
+      <c r="I16" s="5" t="inlineStr">
         <is>
           <t>000007-01, 000007-02, 000007-03, 000007-04, 000007-05, 000007-06, 000007-07</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="J16" s="5" t="inlineStr">
+        <is>
+          <t>Elementary / High School / Teatro: 000007-02, 000007-03, 000007-04</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
         <is>
           <t>000007 Nido de Aguilas</t>
         </is>
@@ -1024,25 +1133,33 @@
         <v>25</v>
       </c>
       <c r="D17" t="n">
+        <v>20</v>
+      </c>
+      <c r="E17" t="n">
         <v>4</v>
       </c>
-      <c r="E17" t="n">
+      <c r="F17" t="n">
         <v>21</v>
       </c>
-      <c r="F17" t="n">
+      <c r="G17" t="n">
         <v>25</v>
       </c>
-      <c r="G17" s="5" t="inlineStr">
+      <c r="H17" s="5" t="inlineStr">
         <is>
           <t>000025-01, 000025-07, 000025-18, 000025-19</t>
         </is>
       </c>
-      <c r="H17" s="5" t="inlineStr">
+      <c r="I17" s="5" t="inlineStr">
         <is>
           <t>000025-04, 000025-08, 000025-10, 000025-12, 000025-13, 000025-17, 000025-20, 000025-21, 000025-22, 000025-23, 000025-24, 000025-27, 000025-28, 000025-29, 000025-32, 000025-33, 000025-34, 000025-35, 000025-36, 000025-37, 000025-38</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="J17" s="5" t="inlineStr">
+        <is>
+          <t>Andén 3-4: 000025-20, 000025-21, 000025-29 · Distrito de lujo: 000025-27, 000025-35, 000025-36 · Anillo Norte/Sur: 000025-37, 000025-38</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
         <is>
           <t>000025 Parque Arauco</t>
         </is>
@@ -1066,18 +1183,26 @@
         <v>4</v>
       </c>
       <c r="E18" t="n">
+        <v>4</v>
+      </c>
+      <c r="F18" t="n">
         <v>0</v>
       </c>
-      <c r="F18" t="n">
+      <c r="G18" t="n">
         <v>12</v>
       </c>
-      <c r="G18" s="5" t="inlineStr">
+      <c r="H18" s="5" t="inlineStr">
         <is>
           <t>000006-01, 000006-02, 000006-04, 000006-05</t>
         </is>
       </c>
-      <c r="H18" s="5" t="inlineStr"/>
-      <c r="I18" t="inlineStr">
+      <c r="I18" s="5" t="inlineStr"/>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
         <is>
           <t>000006 Providencia</t>
         </is>
@@ -1101,18 +1226,26 @@
         <v>5</v>
       </c>
       <c r="E19" t="n">
+        <v>5</v>
+      </c>
+      <c r="F19" t="n">
         <v>0</v>
       </c>
-      <c r="F19" t="n">
+      <c r="G19" t="n">
         <v>1</v>
       </c>
-      <c r="G19" s="5" t="inlineStr">
+      <c r="H19" s="5" t="inlineStr">
         <is>
           <t>000017-04, 000017-05, 000017-06, 000017-07, 000017-08</t>
         </is>
       </c>
-      <c r="H19" s="5" t="inlineStr"/>
-      <c r="I19" t="inlineStr">
+      <c r="I19" s="5" t="inlineStr"/>
+      <c r="J19" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
         <is>
           <t>000017 Renca</t>
         </is>
@@ -1133,31 +1266,41 @@
         <v>2</v>
       </c>
       <c r="D20" t="n">
+        <v>2</v>
+      </c>
+      <c r="E20" t="n">
         <v>0</v>
-      </c>
-      <c r="E20" t="n">
-        <v>2</v>
       </c>
       <c r="F20" t="n">
         <v>2</v>
       </c>
-      <c r="G20" s="5" t="inlineStr"/>
-      <c r="H20" s="5" t="inlineStr">
+      <c r="G20" t="n">
+        <v>2</v>
+      </c>
+      <c r="H20" s="5" t="inlineStr"/>
+      <c r="I20" s="5" t="inlineStr">
         <is>
           <t>000026-01, 000026-02</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
+      <c r="J20" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
         <is>
           <t>000026 UDD</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:I20"/>
-  <mergeCells count="2">
+  <autoFilter ref="A4:K20"/>
+  <mergeCells count="4">
     <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A1:K1"/>
     <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A2:K2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Gabinetes: numerar solo los puntos que están unidos
La celda muestra 1: estos puntos · 2: estos puntos únicamente
cuando varios nodos comparten gabinete. El resto queda en el recuento.

Co-authored-by: anibaloperacionesWes <anibaloperacionesWes@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/Usuarios/acceso_por_empresa/accesos_por_empresa.xlsx
+++ b/reports/Usuarios/acceso_por_empresa/accesos_por_empresa.xlsx
@@ -617,7 +617,7 @@
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
-          <t>1: 000020-01 · 2: 000020-02 · 3: 000020-03 · 4: 000020-04 · 5: 000020-05</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -664,7 +664,7 @@
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>1: 000021-01 · 2: 000021-03 · 3: 000021-04 · 4: 000021-05 · 5: 000021-07</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -707,7 +707,7 @@
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>1: 000031-01 · 2: 000031-02</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -797,7 +797,7 @@
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>1: 000008-01 · 2: 000008-02 · 3: 000008-03 · 4: 000008-04 · 5: 000008-05 · 6: 000008-06 · 7: 000008-07 · 8: 000008-08 · 9: 000008-09 · 10: 000008-10 · 11: 000008-11 · 12: 000008-12 · 13: 000008-13 · 14: 000008-14</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -844,7 +844,7 @@
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>1: 000012-06 · 2: 000012-07 · 3: 000012-08 · 4: 000012-09 · 5: 000012-10 · 6: 000012-11 · 7: 000012-12</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -887,7 +887,7 @@
       </c>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>1: 000027-01 · 2: 000027-02 · 3: 000027-03, 000027-04 · 4: 000027-06 · 5: 000027-07 · 6: 000027-08 · 7: 000027-09</t>
+          <t>1: 000027-03, 000027-04</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -930,7 +930,7 @@
       <c r="I12" s="5" t="inlineStr"/>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>1: 000024-01</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -973,7 +973,7 @@
       <c r="I13" s="5" t="inlineStr"/>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>1: 000022-00</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1020,7 +1020,7 @@
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>1: 000002-01 · 2: 000002-03</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1063,7 +1063,7 @@
       </c>
       <c r="J15" s="5" t="inlineStr">
         <is>
-          <t>1: 000007-01 · 2: 000007-02, 000007-03, 000007-04 · 3: 000007-05 · 4: 000007-06 · 5: 000007-07</t>
+          <t>1: 000007-02, 000007-03, 000007-04</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1110,7 +1110,7 @@
       </c>
       <c r="J16" s="5" t="inlineStr">
         <is>
-          <t>1: 000025-01 · 2: 000025-04 · 3: 000025-07 · 4: 000025-08 · 5: 000025-10 · 6: 000025-12 · 7: 000025-13 · 8: 000025-17 · 9: 000025-18 · 10: 000025-19 · 11: 000025-20, 000025-21, 000025-29 · 12: 000025-22 · 13: 000025-23 · 14: 000025-24 · 15: 000025-27, 000025-35, 000025-36 · 16: 000025-28 · 17: 000025-32 · 18: 000025-33 · 19: 000025-34 · 20: 000025-37, 000025-38</t>
+          <t>1: 000025-20, 000025-21, 000025-29 · 2: 000025-27, 000025-35, 000025-36 · 3: 000025-37, 000025-38</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1153,7 +1153,7 @@
       <c r="I17" s="5" t="inlineStr"/>
       <c r="J17" s="5" t="inlineStr">
         <is>
-          <t>1: 000006-01 · 2: 000006-02 · 3: 000006-04 · 4: 000006-05</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1196,7 +1196,7 @@
       <c r="I18" s="5" t="inlineStr"/>
       <c r="J18" s="5" t="inlineStr">
         <is>
-          <t>1: 000017-04 · 2: 000017-05 · 3: 000017-06 · 4: 000017-07 · 5: 000017-08</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1239,7 +1239,7 @@
       </c>
       <c r="J19" s="5" t="inlineStr">
         <is>
-          <t>1: 000026-01 · 2: 000026-02</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">

</xml_diff>

<commit_message>
Regenerar reporte de accesos con columna SIM 4G
Co-authored-by: anibaloperacionesWes <anibaloperacionesWes@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/Usuarios/acceso_por_empresa/accesos_por_empresa.xlsx
+++ b/reports/Usuarios/acceso_por_empresa/accesos_por_empresa.xlsx
@@ -1,33 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CPA control" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Puntos" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="000020 AGUNSA" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="000021 CDUC" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="000031 Club Providencia" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="000009 COPEC" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="000008 CORMUP" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="000012 DERCO" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="000027 Fundo Zapallar" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="000024 La Reina" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="000022 Las Condes" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="000002 Lo valledor" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="000007 Nido de Aguilas" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="000025 Parque Arauco" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="000006 Providencia" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="000017 Renca" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="000026 UDD" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Resumen" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="CPA control" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Puntos" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="000020 AGUNSA" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="000021 CDUC" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="000031 Club Providencia" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="000009 COPEC" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="000008 CORMUP" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="000012 DERCO" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="000027 Fundo Zapallar" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="000024 La Reina" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="000022 Las Condes" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="000002 Lo valledor" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="000007 Nido de Aguilas" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="000025 Parque Arauco" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="000006 Providencia" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="000017 Renca" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="000026 UDD" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$4:$K$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$4:$L$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CPA control'!$A$4:$F$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Puntos'!$A$4:$F$104</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'000020 AGUNSA'!$A$4:$H$19</definedName>
@@ -53,7 +53,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -74,6 +74,10 @@
       <b val="1"/>
       <color rgb="00375623"/>
       <sz val="14"/>
+    </font>
+    <font>
+      <color rgb="00555555"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="6">
@@ -116,7 +120,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -127,6 +131,7 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -492,14 +497,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K19"/>
+  <dimension ref="A1:L19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="36" customWidth="1" min="8" max="8"/>
@@ -516,12 +521,13 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Generado 28/08/2026 09:12 hora Chile · se omite personal WES (@wes.cl); se incluye go.salass@gmail.com. CPA = monitoreo con control (horarios programados Drive). Solo monitoreo = punto activo sin CPA. Gabinetes: puntos en el mismo gabinete cuentan como 1.</t>
-        </is>
-      </c>
-    </row>
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>Generado 28/08/2026 09:12 hora Chile · se omite personal WES (@wes.cl); se incluye go.salass@gmail.com. CPA = monitoreo con control (horarios programados Drive). Solo monitoreo = punto activo sin CPA. Gabinetes: puntos en el mismo gabinete cuentan como 1. SIM 4G: igual que gabinetes, salvo internet del cliente (AGUNSA, Nido, Lo Valledor P1).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
@@ -545,35 +551,40 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
+          <t>sim_4g</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
           <t>puntos_CPA</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>puntos_solo_monitoreo</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>usuarios_con_acceso</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>ids_CPA</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>ids_solo_monitoreo</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>mismo_gabinete</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>hoja</t>
         </is>
@@ -596,31 +607,37 @@
       <c r="D5" t="n">
         <v>5</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>0
+Internet AGUNSA (la empresa alimenta los 5 puntos)</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
         <v>1</v>
       </c>
-      <c r="F5" t="n">
+      <c r="G5" t="n">
         <v>4</v>
       </c>
-      <c r="G5" t="n">
+      <c r="H5" t="n">
         <v>15</v>
       </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="I5" s="5" t="inlineStr">
         <is>
           <t>000020-02</t>
         </is>
       </c>
-      <c r="I5" s="5" t="inlineStr">
+      <c r="J5" s="5" t="inlineStr">
         <is>
           <t>000020-01, 000020-03, 000020-04, 000020-05</t>
         </is>
       </c>
-      <c r="J5" s="5" t="inlineStr">
+      <c r="K5" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>000020 AGUNSA</t>
         </is>
@@ -643,31 +660,36 @@
       <c r="D6" t="n">
         <v>5</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
         <v>2</v>
       </c>
-      <c r="F6" t="n">
+      <c r="G6" t="n">
         <v>3</v>
       </c>
-      <c r="G6" t="n">
+      <c r="H6" t="n">
         <v>12</v>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="I6" s="5" t="inlineStr">
         <is>
           <t>000021-01, 000021-03</t>
         </is>
       </c>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="J6" s="5" t="inlineStr">
         <is>
           <t>000021-04, 000021-05, 000021-07</t>
         </is>
       </c>
-      <c r="J6" s="5" t="inlineStr">
+      <c r="K6" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>000021 CDUC</t>
         </is>
@@ -690,27 +712,32 @@
       <c r="D7" t="n">
         <v>2</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
         <v>0</v>
       </c>
-      <c r="F7" t="n">
+      <c r="G7" t="n">
         <v>2</v>
       </c>
-      <c r="G7" t="n">
+      <c r="H7" t="n">
         <v>6</v>
       </c>
-      <c r="H7" s="5" t="inlineStr"/>
-      <c r="I7" s="5" t="inlineStr">
+      <c r="I7" s="5" t="inlineStr"/>
+      <c r="J7" s="5" t="inlineStr">
         <is>
           <t>000031-01, 000031-02</t>
         </is>
       </c>
-      <c r="J7" s="5" t="inlineStr">
+      <c r="K7" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>000031 Club Providencia</t>
         </is>
@@ -733,27 +760,33 @@
       <c r="D8" t="n">
         <v>4</v>
       </c>
-      <c r="E8" t="n">
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>4
+1: 000009-00, 000009-01 · 2: 000009-02, 000009-05, 000009-06 · 3: 000009-03, 000009-04, 000009-09, 000009-10 · 4: 000009-08, 000009-11</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
         <v>0</v>
       </c>
-      <c r="F8" t="n">
+      <c r="G8" t="n">
         <v>11</v>
       </c>
-      <c r="G8" t="n">
+      <c r="H8" t="n">
         <v>6</v>
       </c>
-      <c r="H8" s="5" t="inlineStr"/>
-      <c r="I8" s="5" t="inlineStr">
+      <c r="I8" s="5" t="inlineStr"/>
+      <c r="J8" s="5" t="inlineStr">
         <is>
           <t>000009-00, 000009-01, 000009-02, 000009-03, 000009-04, 000009-05, 000009-06, 000009-08, 000009-09, 000009-10, 000009-11</t>
         </is>
       </c>
-      <c r="J8" s="5" t="inlineStr">
+      <c r="K8" s="5" t="inlineStr">
         <is>
           <t>1: 000009-00, 000009-01 · 2: 000009-02, 000009-05, 000009-06 · 3: 000009-03, 000009-04, 000009-09, 000009-10 · 4: 000009-08, 000009-11</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>000009 COPEC</t>
         </is>
@@ -776,31 +809,36 @@
       <c r="D9" t="n">
         <v>14</v>
       </c>
-      <c r="E9" t="n">
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
         <v>11</v>
       </c>
-      <c r="F9" t="n">
+      <c r="G9" t="n">
         <v>3</v>
       </c>
-      <c r="G9" t="n">
+      <c r="H9" t="n">
         <v>2</v>
       </c>
-      <c r="H9" s="5" t="inlineStr">
+      <c r="I9" s="5" t="inlineStr">
         <is>
           <t>000008-01, 000008-03, 000008-04, 000008-05, 000008-06, 000008-07, 000008-09, 000008-10, 000008-11, 000008-12, 000008-14</t>
         </is>
       </c>
-      <c r="I9" s="5" t="inlineStr">
+      <c r="J9" s="5" t="inlineStr">
         <is>
           <t>000008-02, 000008-08, 000008-13</t>
         </is>
       </c>
-      <c r="J9" s="5" t="inlineStr">
+      <c r="K9" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>000008 CORMUP</t>
         </is>
@@ -823,31 +861,36 @@
       <c r="D10" t="n">
         <v>7</v>
       </c>
-      <c r="E10" t="n">
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
         <v>1</v>
       </c>
-      <c r="F10" t="n">
+      <c r="G10" t="n">
         <v>6</v>
       </c>
-      <c r="G10" t="n">
+      <c r="H10" t="n">
         <v>1</v>
       </c>
-      <c r="H10" s="5" t="inlineStr">
+      <c r="I10" s="5" t="inlineStr">
         <is>
           <t>000012-06</t>
         </is>
       </c>
-      <c r="I10" s="5" t="inlineStr">
+      <c r="J10" s="5" t="inlineStr">
         <is>
           <t>000012-07, 000012-08, 000012-09, 000012-10, 000012-11, 000012-12</t>
         </is>
       </c>
-      <c r="J10" s="5" t="inlineStr">
+      <c r="K10" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>000012 DERCO</t>
         </is>
@@ -870,27 +913,33 @@
       <c r="D11" t="n">
         <v>7</v>
       </c>
-      <c r="E11" t="n">
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>7
+1: 000027-03, 000027-04</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
         <v>0</v>
       </c>
-      <c r="F11" t="n">
+      <c r="G11" t="n">
         <v>8</v>
       </c>
-      <c r="G11" t="n">
+      <c r="H11" t="n">
         <v>7</v>
       </c>
-      <c r="H11" s="5" t="inlineStr"/>
-      <c r="I11" s="5" t="inlineStr">
+      <c r="I11" s="5" t="inlineStr"/>
+      <c r="J11" s="5" t="inlineStr">
         <is>
           <t>000027-01, 000027-02, 000027-03, 000027-04, 000027-06, 000027-07, 000027-08, 000027-09</t>
         </is>
       </c>
-      <c r="J11" s="5" t="inlineStr">
+      <c r="K11" s="5" t="inlineStr">
         <is>
           <t>1: 000027-03, 000027-04</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="L11" t="inlineStr">
         <is>
           <t>000027 Fundo Zapallar</t>
         </is>
@@ -913,27 +962,32 @@
       <c r="D12" t="n">
         <v>1</v>
       </c>
-      <c r="E12" t="n">
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
         <v>1</v>
       </c>
-      <c r="F12" t="n">
+      <c r="G12" t="n">
         <v>0</v>
       </c>
-      <c r="G12" t="n">
+      <c r="H12" t="n">
         <v>2</v>
       </c>
-      <c r="H12" s="5" t="inlineStr">
+      <c r="I12" s="5" t="inlineStr">
         <is>
           <t>000024-01</t>
         </is>
       </c>
-      <c r="I12" s="5" t="inlineStr"/>
-      <c r="J12" s="5" t="inlineStr">
+      <c r="J12" s="5" t="inlineStr"/>
+      <c r="K12" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="L12" t="inlineStr">
         <is>
           <t>000024 La Reina</t>
         </is>
@@ -956,27 +1010,32 @@
       <c r="D13" t="n">
         <v>1</v>
       </c>
-      <c r="E13" t="n">
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
         <v>1</v>
       </c>
-      <c r="F13" t="n">
+      <c r="G13" t="n">
         <v>0</v>
       </c>
-      <c r="G13" t="n">
+      <c r="H13" t="n">
         <v>1</v>
       </c>
-      <c r="H13" s="5" t="inlineStr">
+      <c r="I13" s="5" t="inlineStr">
         <is>
           <t>000022-00</t>
         </is>
       </c>
-      <c r="I13" s="5" t="inlineStr"/>
-      <c r="J13" s="5" t="inlineStr">
+      <c r="J13" s="5" t="inlineStr"/>
+      <c r="K13" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>000022 Las Condes</t>
         </is>
@@ -999,31 +1058,37 @@
       <c r="D14" t="n">
         <v>2</v>
       </c>
-      <c r="E14" t="n">
-        <v>1</v>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>1
+P1 / Placa 1 (000002-01): problema</t>
+        </is>
       </c>
       <c r="F14" t="n">
         <v>1</v>
       </c>
       <c r="G14" t="n">
+        <v>1</v>
+      </c>
+      <c r="H14" t="n">
         <v>6</v>
       </c>
-      <c r="H14" s="5" t="inlineStr">
+      <c r="I14" s="5" t="inlineStr">
         <is>
           <t>000002-01</t>
         </is>
       </c>
-      <c r="I14" s="5" t="inlineStr">
+      <c r="J14" s="5" t="inlineStr">
         <is>
           <t>000002-03</t>
         </is>
       </c>
-      <c r="J14" s="5" t="inlineStr">
+      <c r="K14" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="L14" t="inlineStr">
         <is>
           <t>000002 Lo valledor</t>
         </is>
@@ -1046,27 +1111,33 @@
       <c r="D15" t="n">
         <v>5</v>
       </c>
-      <c r="E15" t="n">
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>2
+Internet cliente: Estanque B, Teatro, High School, Elementary, Pozo Profundo</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
         <v>0</v>
       </c>
-      <c r="F15" t="n">
+      <c r="G15" t="n">
         <v>7</v>
       </c>
-      <c r="G15" t="n">
+      <c r="H15" t="n">
         <v>4</v>
       </c>
-      <c r="H15" s="5" t="inlineStr"/>
-      <c r="I15" s="5" t="inlineStr">
+      <c r="I15" s="5" t="inlineStr"/>
+      <c r="J15" s="5" t="inlineStr">
         <is>
           <t>000007-01, 000007-02, 000007-03, 000007-04, 000007-05, 000007-06, 000007-07</t>
         </is>
       </c>
-      <c r="J15" s="5" t="inlineStr">
+      <c r="K15" s="5" t="inlineStr">
         <is>
           <t>1: 000007-02, 000007-03, 000007-04</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="L15" t="inlineStr">
         <is>
           <t>000007 Nido de Aguilas</t>
         </is>
@@ -1089,31 +1160,37 @@
       <c r="D16" t="n">
         <v>20</v>
       </c>
-      <c r="E16" t="n">
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>20
+1: 000025-20, 000025-21, 000025-29 · 2: 000025-27, 000025-35, 000025-36 · 3: 000025-37, 000025-38</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
         <v>4</v>
       </c>
-      <c r="F16" t="n">
+      <c r="G16" t="n">
         <v>21</v>
       </c>
-      <c r="G16" t="n">
+      <c r="H16" t="n">
         <v>25</v>
       </c>
-      <c r="H16" s="5" t="inlineStr">
+      <c r="I16" s="5" t="inlineStr">
         <is>
           <t>000025-01, 000025-07, 000025-18, 000025-19</t>
         </is>
       </c>
-      <c r="I16" s="5" t="inlineStr">
+      <c r="J16" s="5" t="inlineStr">
         <is>
           <t>000025-04, 000025-08, 000025-10, 000025-12, 000025-13, 000025-17, 000025-20, 000025-21, 000025-22, 000025-23, 000025-24, 000025-27, 000025-28, 000025-29, 000025-32, 000025-33, 000025-34, 000025-35, 000025-36, 000025-37, 000025-38</t>
         </is>
       </c>
-      <c r="J16" s="5" t="inlineStr">
+      <c r="K16" s="5" t="inlineStr">
         <is>
           <t>1: 000025-20, 000025-21, 000025-29 · 2: 000025-27, 000025-35, 000025-36 · 3: 000025-37, 000025-38</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
+      <c r="L16" t="inlineStr">
         <is>
           <t>000025 Parque Arauco</t>
         </is>
@@ -1136,27 +1213,32 @@
       <c r="D17" t="n">
         <v>4</v>
       </c>
-      <c r="E17" t="n">
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
         <v>4</v>
       </c>
-      <c r="F17" t="n">
+      <c r="G17" t="n">
         <v>0</v>
       </c>
-      <c r="G17" t="n">
+      <c r="H17" t="n">
         <v>12</v>
       </c>
-      <c r="H17" s="5" t="inlineStr">
+      <c r="I17" s="5" t="inlineStr">
         <is>
           <t>000006-01, 000006-02, 000006-04, 000006-05</t>
         </is>
       </c>
-      <c r="I17" s="5" t="inlineStr"/>
-      <c r="J17" s="5" t="inlineStr">
+      <c r="J17" s="5" t="inlineStr"/>
+      <c r="K17" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr">
+      <c r="L17" t="inlineStr">
         <is>
           <t>000006 Providencia</t>
         </is>
@@ -1179,27 +1261,32 @@
       <c r="D18" t="n">
         <v>5</v>
       </c>
-      <c r="E18" t="n">
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
         <v>5</v>
       </c>
-      <c r="F18" t="n">
+      <c r="G18" t="n">
         <v>0</v>
       </c>
-      <c r="G18" t="n">
+      <c r="H18" t="n">
         <v>1</v>
       </c>
-      <c r="H18" s="5" t="inlineStr">
+      <c r="I18" s="5" t="inlineStr">
         <is>
           <t>000017-04, 000017-05, 000017-06, 000017-07, 000017-08</t>
         </is>
       </c>
-      <c r="I18" s="5" t="inlineStr"/>
-      <c r="J18" s="5" t="inlineStr">
+      <c r="J18" s="5" t="inlineStr"/>
+      <c r="K18" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr">
+      <c r="L18" t="inlineStr">
         <is>
           <t>000017 Renca</t>
         </is>
@@ -1222,39 +1309,42 @@
       <c r="D19" t="n">
         <v>2</v>
       </c>
-      <c r="E19" t="n">
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
         <v>0</v>
-      </c>
-      <c r="F19" t="n">
-        <v>2</v>
       </c>
       <c r="G19" t="n">
         <v>2</v>
       </c>
-      <c r="H19" s="5" t="inlineStr"/>
-      <c r="I19" s="5" t="inlineStr">
+      <c r="H19" t="n">
+        <v>2</v>
+      </c>
+      <c r="I19" s="5" t="inlineStr"/>
+      <c r="J19" s="5" t="inlineStr">
         <is>
           <t>000026-01, 000026-02</t>
         </is>
       </c>
-      <c r="J19" s="5" t="inlineStr">
+      <c r="K19" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
+      <c r="L19" t="inlineStr">
         <is>
           <t>000026 UDD</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:K20"/>
-  <mergeCells count="4">
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A2:I2"/>
-    <mergeCell ref="A2:K2"/>
+  <autoFilter ref="A4:L19"/>
+  <mergeCells count="2">
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A1:L1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>